<commit_message>
feat: schema fixes + open tasks in context + DM history
Schema fixes (Excel/Notion alignment):
- Backlog: Status "To do"→"A fazer", Priority "1. Alta"→"Alta" etc.
- Lembretes: title field "Reminder"→"Texto"
- Studio Log: Owner select→multi_select
- Content Calendar: status values→lowercase (raw idea, ideation, etc.)
- Para Discutir: add entity_ref relation support (project, event, etc.)
- System prompt: fix to_discuss estado (Discutido), decisions estado, prioridade values

Context improvements:
- Open tasks (sender's) now included in every assistant message
- DM handler: add message history + lastBotReplies (parity with group)
- Shared history module (src/bot/history.ts) used by both index + dm

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/notion-db-config.xlsx
+++ b/docs/notion-db-config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madsi\Claude_stuff\Code\Haven-VA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EAB967B-3977-44D9-90B1-7F7F6F6B75DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C32DF7AF-C1D8-4463-9F2F-248F13135629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3948" yWindow="12852" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Backlog" sheetId="1" r:id="rId1"/>
@@ -22,14 +22,16 @@
     <sheet name="Projetos" sheetId="8" r:id="rId7"/>
     <sheet name="Eventos" sheetId="9" r:id="rId8"/>
     <sheet name="Listas" sheetId="10" r:id="rId9"/>
-    <sheet name="Content Calendar" sheetId="5" r:id="rId10"/>
+    <sheet name="Studio Log" sheetId="11" r:id="rId10"/>
+    <sheet name="Founder Focus" sheetId="12" r:id="rId11"/>
+    <sheet name="Content Calendar" sheetId="5" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="108">
   <si>
     <t>Propriedade</t>
   </si>
@@ -296,6 +298,63 @@
   </si>
   <si>
     <t>Fechada</t>
+  </si>
+  <si>
+    <t>Series</t>
+  </si>
+  <si>
+    <t>Haven About/Benefits/Community | Pilates Educational | Filler Studio/Motivational/Relatable/Funny | Customer Highlight | Instructor Highlight | Funny &amp; Relatable | Day to day | About us</t>
+  </si>
+  <si>
+    <t>Caption</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>Script</t>
+  </si>
+  <si>
+    <t>Post URL</t>
+  </si>
+  <si>
+    <t>Clips</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Inspo video</t>
+  </si>
+  <si>
+    <t>Recording date</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Active ad</t>
+  </si>
+  <si>
+    <t>Haven | Ad</t>
+  </si>
+  <si>
+    <t>Founder</t>
+  </si>
+  <si>
+    <t>Foco operacional</t>
+  </si>
+  <si>
+    <t>bot cria nome com base no que escrevemos no foco operacional</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Tags</t>
   </si>
 </sst>
 </file>
@@ -673,7 +732,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -681,7 +740,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -695,7 +754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -709,7 +768,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -723,7 +782,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -737,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -751,7 +810,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -765,7 +824,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -779,7 +838,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>40</v>
       </c>
@@ -793,7 +852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -807,7 +866,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -821,7 +880,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -835,7 +894,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -849,7 +908,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -863,7 +922,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -877,7 +936,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -900,9 +959,152 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BA722BE-9022-4AB0-BEFD-91B2D74B1940}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="4" width="15.69921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29BEBF89-D52C-4C5B-8C13-A9DBF20C6AAA}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="4" width="17.296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -910,7 +1112,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -924,7 +1126,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -938,7 +1140,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -952,7 +1154,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -966,7 +1168,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -980,7 +1182,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>61</v>
       </c>
@@ -992,6 +1194,92 @@
       </c>
       <c r="D6" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1005,7 +1293,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1013,7 +1301,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1027,7 +1315,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>35</v>
       </c>
@@ -1041,7 +1329,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -1055,7 +1343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>38</v>
       </c>
@@ -1069,7 +1357,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1083,7 +1371,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -1186,7 +1474,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1194,7 +1482,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1208,7 +1496,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -1222,7 +1510,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1236,7 +1524,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -1250,7 +1538,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1264,7 +1552,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -1278,7 +1566,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>48</v>
       </c>
@@ -1292,7 +1580,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1306,7 +1594,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1381,7 +1669,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1389,7 +1677,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1403,7 +1691,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -1417,7 +1705,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1431,7 +1719,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>52</v>
       </c>
@@ -1445,7 +1733,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -1459,7 +1747,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1548,7 +1836,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1556,7 +1844,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1570,7 +1858,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1584,7 +1872,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>63</v>
       </c>
@@ -1598,7 +1886,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1612,7 +1900,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1626,7 +1914,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -1640,7 +1928,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -1681,7 +1969,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1689,7 +1977,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1703,7 +1991,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1717,7 +2005,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>66</v>
       </c>
@@ -1731,7 +2019,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1745,7 +2033,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1759,7 +2047,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -1773,7 +2061,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -1839,7 +2127,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1847,7 +2135,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1861,7 +2149,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1875,7 +2163,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1954,7 +2242,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -1962,7 +2250,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1976,7 +2264,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1990,7 +2278,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2004,7 +2292,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2072,7 +2360,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.796875" customWidth="1"/>
     <col min="2" max="2" width="14.796875" customWidth="1"/>
@@ -2080,7 +2368,7 @@
     <col min="4" max="4" width="28.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2094,7 +2382,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -2108,7 +2396,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -2122,7 +2410,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>88</v>
       </c>
@@ -2136,7 +2424,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>43</v>
       </c>

</xml_diff>